<commit_message>
Actualizar alcance, bitácora e informe con resultados recientes
</commit_message>
<xml_diff>
--- a/tarea1-gestor-contrasenas/docs/red-team/04-bitacora-planilla.xlsx
+++ b/tarea1-gestor-contrasenas/docs/red-team/04-bitacora-planilla.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R9a77c3f69c384289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R26bb634893fe44a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1291,6 +1291,141 @@
         <x:v>El usuario declaró que el carácter era a; las capturas muestran un carácter oculto y la misma ruta abierta. 01–03 son un intento previo descartado por error de tecla. Riesgo condicionado a obtener el archivo cifrado; sin descifrado externo ni severidad asignada.</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="95" customHeight="1">
+      <x:c r="A29" s="7" t="d">
+        <x:v>2026-10-30T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B29" s="9"/>
+      <x:c r="C29" s="6" t="str">
+        <x:v>Red Team / RT-P11 revisión del repositorio</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="str">
+        <x:v>Equipo Red Team; firma pendiente</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="str">
+        <x:v>Revisar archivos versionados, 87 commits locales y evidencias Red Team aún sin versionar en busca de secretos y configuración insegura.</x:v>
+      </x:c>
+      <x:c r="F29" s="6" t="str">
+        <x:v>Git, búsqueda de patrones sin imprimir valores, revisión manual de plantillas, .gitignore, Dockerfile y compose.</x:v>
+      </x:c>
+      <x:c r="G29" s="6" t="str">
+        <x:v>Sin secreto operativo confirmado en historial. Tres JWS vencidos en nueve archivos locales sin versionar; RT-P11-revision-repositorio.md y evidencias/RT-P11/.</x:v>
+      </x:c>
+      <x:c r="H29" s="6" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="I29" s="6" t="str">
+        <x:v>Revisión de solo lectura. No se enviaron solicitudes ni se inspeccionó el archivo red-team.rar. Sanear JWS antes de publicar. Hora UTC de actividad no registrada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="95" customHeight="1">
+      <x:c r="A30" s="7" t="d">
+        <x:v>2026-10-30T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B30" s="9"/>
+      <x:c r="C30" s="6" t="str">
+        <x:v>Red Team / RT-P12 error de maestra</x:v>
+      </x:c>
+      <x:c r="D30" s="6" t="str">
+        <x:v>Usuario ejecutor; firma pendiente</x:v>
+      </x:c>
+      <x:c r="E30" s="6" t="str">
+        <x:v>Intentar abrir una bóveda con maestra incorrecta y repetir con un marcador ficticio; revisar interfaz, evento de auditoría y archivos locales de auditoría. El 31/10: importar una copia ficticia inexistente con contraseña de transporte ficticia. Crear copia cifrada de bóveda vacía e intentar importarla con contraseña de transporte ficticia incorrecta. Intentar abrir bóveda con maestra correcta y código TOTP ficticio inválido.</x:v>
+      </x:c>
+      <x:c r="F30" s="6" t="str">
+        <x:v>Cliente gestor; API de eventos; revisión de código Rust; búsqueda local acotada.</x:v>
+      </x:c>
+      <x:c r="G30" s="6" t="str">
+        <x:v>Rechazo genérico; eventos 94 y 95 de intento_fallido_maestra con firma válida; marcador ausente en auditoria.json y ultimo.txt. RT-P12-error-maestra-sin-filtracion.md; evidencias/RT-P12/01, 02 y 03-eventos-auditoria.json; SHA256SUMS.txt. Verificación adicional: marcador ficticio ausente en logs recientes del backend; evidencias/RT-P12/04-verificacion-logs-backend.txt. El usuario corroboró NO APARECE en Linux; evidencia 05-consulta-logs-usuario.png. Error de archivo no encontrado sin revelar la contraseña de transporte; evidencia 06-importacion-archivo-inexistente.png. Rechazo genérico sin revelar contraseña; evidencias 07-copia-cifrada-guardada.png y 08-transporte-incorrecto.png. Código TOTP inválido, sin exposición del secreto; evidencia 09-totp-invalido.png.</x:v>
+      </x:c>
+      <x:c r="H30" s="6" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="I30" s="6" t="str">
+        <x:v>RT-10 parcial. No se observó filtración en este error ni en su evento; no se revisaron exhaustivamente otros errores, logs o memoria. Capturas del 30/10 local; hora UTC de actividad no registrada. Logs de control-central revisados desde 31/10 02:00 UTC; consulta 02:40 UTC. Otros servicios y rutas no revisados. Archivo de prueba no creado; marcador ausente en auditoria.json y ultimo.txt. Este caso no prueba una contraseña de transporte incorrecta. Copia .gex presente (74 bytes); marcador ausente en archivos locales de auditoría. RT-10 aún parcial. RT-10 cerrado para cuatro caminos de error; otros errores y memoria no evaluados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" t="d">
+        <x:v>2026-10-31T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B31"/>
+      <x:c r="C31" t="str">
+        <x:v>Red Team / RT-P13 sqlmap login</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>Usuario ejecutor; firma pendiente</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>Comprobar inyección SQL en el parámetro JSON email de POST /api/users/login con datos ficticios.</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>sqlmap 1.10.11.1#dev; --risk=1 --level=1 --technique=BE --threads=1 --delay=0.2 --ignore-code=401; límite 180 s.</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Primera ejecución detenida por 401. Segunda ejecución completa: sqlmap no identificó inyección en email; 36 respuestas 401. RT-P13-sqlmap-login.md; evidencias/RT-P13/01 y 02; SHA256SUMS.txt.</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>Resultado limitado al campo email y configuración usada; no descarta inyección en otras rutas. RT-03 cubierto por RT-P04/H01 (lectura de auditoría sin sesión), no por este resultado negativo. Ejecución desde VM Linux; hora UTC de las capturas 03:40 y 03:42, equivalente al 31/10 local. No se verificó por separado el archivo de salida de sqlmap.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="A32" t="d">
+        <x:v>2026-10-31T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B32"/>
+      <x:c r="C32" t="str">
+        <x:v>Red Team / RT-P14 correo Mailpit</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>Usuario ejecutor; firma pendiente</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>Enviar un único correo ficticio por SMTP al receptor de laboratorio y comprobar que aparece en Mailpit.</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Swaks 20240103.0 contra 192.168.77.10:1025; interfaz Mailpit por túnel SSH al puerto 8025.</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>SMTP devolvió 250 2.0.0 Ok: queued; Mailpit mostró el mensaje. RT-P14-correo-mailpit.md; evidencias/RT-P14/01 y 02; SHA256SUMS.txt.</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>Comprobación parcial de RT-04. Mailpit es un receptor de pruebas; no se demostró relay a Internet, SPF/DKIM defectuoso ni suplantación de un servidor real. Remitente coincide con el valor predeterminado de la aplicación. Hora UTC de envío observada: 12:54:40; fecha local 31/10. No se enviaron correos reales.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="A33" t="d">
+        <x:v>2026-10-31T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B33"/>
+      <x:c r="C33" t="str">
+        <x:v>Red Team / RT-05 revisión documental</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>Equipo Red Team; firma pendiente</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>Revisar la declaración del Blue Team sobre la ausencia de TLS y el riesgo residual R05.</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Lectura de docs/00-arquitectura-c4.md y docs/03-Analisis-Riesgos.md; hashes SHA-256.</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>La documentación declara HTTP sin TLS en cliente a API y aceptación de R05. RT-05-revision-documental-tls.md; evidencias/RT-05/01-fuentes-documentales.txt.</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>Solo análisis documental. No se ejecutó MITM, interceptación, alteración de tráfico ni prueba de certificados. No se cuenta como prueba ejecutada ni como hallazgo nuevo. Hora UTC de revisión no registrada.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>